<commit_message>
stable refactoring finished first hand
</commit_message>
<xml_diff>
--- a/preprocessing/oversampling.xlsx
+++ b/preprocessing/oversampling.xlsx
@@ -112,7 +112,7 @@
     <t xml:space="preserve">cropped_0001_label_wmLYCo2j_1440_1440.png</t>
   </si>
   <si>
-    <t xml:space="preserve">cropped_00000002_4_480_960.png </t>
+    <t xml:space="preserve">cropped_00000002_4_480_960.png</t>
   </si>
   <si>
     <t xml:space="preserve">cropped_00000002_4_2400_960.png</t>
@@ -166,7 +166,7 @@
     <t xml:space="preserve">cropped_0004_label_1XDZxhBC_0_1440.png</t>
   </si>
   <si>
-    <t xml:space="preserve">cropped_0004_label_5caRcr55_1920_960.png **</t>
+    <t xml:space="preserve">cropped_0004_label_5caRcr55_1920_960.png</t>
   </si>
   <si>
     <t xml:space="preserve">cropped_0004_label_FcjmsocM_960_480.png</t>

</xml_diff>